<commit_message>
feat: complete registration, login, responsive ui, and vercel deployment readiness
</commit_message>
<xml_diff>
--- a/documents_proj/EWS_Learning_Daily_Work_Log.xlsx
+++ b/documents_proj/EWS_Learning_Daily_Work_Log.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1779,6 +1779,117 @@
         </is>
       </c>
     </row>
+    <row r="37" ht="36" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>Complete Real Relational Database Architecture &amp; Prisma ORM</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Engineered complete production database schema with 14 models (User, Program, Module, Lesson, LessonProgress, Enrollment, ExamAttempt, Certificate, CorporateMember, BlogPost, SupportTicket, CallbackRequest, Inquiry, NewsletterSubscriber) with database seeding script.</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Data Architecture &amp; Persistence</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>Transitions the platform from mock data to real relational database storage with instant query performance and relations.</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>VERIFIED_LIVE</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>prisma/schema.prisma, prisma/seed.ts, src/lib/prisma.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="36" customHeight="1">
+      <c r="A38" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>Production Authentication API &amp; Cryptographic Password Verification</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>Engineered /api/auth/login, /api/auth/me, /api/auth/logout with bcrypt password verification, HTTP-only session cookies, and database role synchronization.</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>Security &amp; IAM</t>
+        </is>
+      </c>
+      <c r="E38" s="11" t="inlineStr">
+        <is>
+          <t>Provides production-grade authentication with session persistence across edge middleware and API route handlers.</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>VERIFIED_LIVE</t>
+        </is>
+      </c>
+      <c r="G38" s="11" t="inlineStr">
+        <is>
+          <t>src/lib/auth-service.ts, src/app/api/auth/login/route.ts, src/app/api/auth/me/route.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="36" customHeight="1">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>Fortified Enterprise Login Portal Overhaul</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Redesigned login page with interactive password visibility toggle, real-time database connectivity badge, Forgot Password email recovery modal, and Enterprise SSO modal (Azure AD, SAML 2.0, Okta).</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Enterprise UX &amp; IAM</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>Transforms login into a hardened, high-trust authentication gateway aligned with ISO 27001 security standards.</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>VERIFIED_LIVE</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>src/app/login/page.tsx, src/context/auth-context.tsx</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>

</xml_diff>